<commit_message>
Sync process templates, checklist grouping, and timeline calculations across backend, database schema, and frontend UI.
</commit_message>
<xml_diff>
--- a/document/08_PMI-เครื่องติดแสตมป์_ออฟ โอ๋ อ้วน.xlsx
+++ b/document/08_PMI-เครื่องติดแสตมป์_ออฟ โอ๋ อ้วน.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milln\CWN Work\Project-Tracking\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D4D619-BD4D-4D5A-9ABC-4E9EA96925B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD98A2E9-87DE-47A0-A1E5-1BC91EF3D901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="713" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="172">
   <si>
     <t>📊 EXECUTIVE PROJECT DASHBOARD (ระบบวิเคราะห์และติดตามสถานะโครงการ)</t>
   </si>
@@ -554,6 +554,9 @@
   </si>
   <si>
     <t>ref</t>
+  </si>
+  <si>
+    <t>check</t>
   </si>
 </sst>
 </file>
@@ -1075,6 +1078,57 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1093,59 +1147,8 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1420,14 +1423,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="60"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7">
@@ -1439,14 +1442,14 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="64" t="s">
+      <c r="A3" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="60"/>
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="77"/>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7">
@@ -1509,14 +1512,14 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="65" t="s">
+      <c r="A8" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="60"/>
+      <c r="B8" s="79"/>
+      <c r="C8" s="79"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="79"/>
+      <c r="F8" s="77"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7">
@@ -1562,21 +1565,21 @@
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="60"/>
+      <c r="B12" s="79"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="77"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="59" t="s">
+      <c r="A13" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="60"/>
+      <c r="B13" s="77"/>
       <c r="C13" s="20" t="s">
         <v>21</v>
       </c>
@@ -1586,10 +1589,10 @@
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="60"/>
+      <c r="B14" s="77"/>
       <c r="C14" s="10" t="s">
         <v>23</v>
       </c>
@@ -1599,10 +1602,10 @@
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="59" t="s">
+      <c r="A15" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="60"/>
+      <c r="B15" s="77"/>
       <c r="C15" s="25" t="s">
         <v>25</v>
       </c>
@@ -1612,10 +1615,10 @@
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="76" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="60"/>
+      <c r="B16" s="77"/>
       <c r="C16" s="28" t="s">
         <v>27</v>
       </c>
@@ -1634,14 +1637,14 @@
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="60"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="77"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7">
@@ -2124,7 +2127,7 @@
     <col min="9" max="9" width="56.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="13.2">
       <c r="A1" s="3" t="s">
         <v>59</v>
       </c>
@@ -2132,7 +2135,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" ht="13.2">
       <c r="A2" s="37" t="s">
         <v>61</v>
       </c>
@@ -2159,6 +2162,9 @@
       <c r="G4" t="s">
         <v>169</v>
       </c>
+      <c r="H4" t="s">
+        <v>171</v>
+      </c>
       <c r="I4" t="s">
         <v>163</v>
       </c>
@@ -2166,7 +2172,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" ht="13.2">
       <c r="A5" s="38" t="s">
         <v>29</v>
       </c>
@@ -2198,7 +2204,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" ht="13.8">
       <c r="A6" s="39"/>
       <c r="B6" s="40" t="s">
         <v>70</v>
@@ -2216,7 +2222,7 @@
       <c r="I6" s="40"/>
       <c r="J6" s="46"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" ht="13.8">
       <c r="A7" s="39" t="s">
         <v>35</v>
       </c>
@@ -2249,7 +2255,7 @@
       </c>
       <c r="J7" s="46"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" ht="13.8">
       <c r="A8" s="39" t="s">
         <v>35</v>
       </c>
@@ -2283,7 +2289,7 @@
       </c>
       <c r="J8" s="46"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" ht="13.8">
       <c r="A9" s="39" t="s">
         <v>35</v>
       </c>
@@ -2317,7 +2323,7 @@
       </c>
       <c r="J9" s="46"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" ht="13.8">
       <c r="A10" s="39" t="s">
         <v>35</v>
       </c>
@@ -2351,7 +2357,7 @@
       </c>
       <c r="J10" s="46"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" ht="13.8">
       <c r="A11" s="39" t="s">
         <v>35</v>
       </c>
@@ -2385,7 +2391,7 @@
       </c>
       <c r="J11" s="46"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" ht="13.8">
       <c r="A12" s="39" t="s">
         <v>41</v>
       </c>
@@ -2419,7 +2425,7 @@
       </c>
       <c r="J12" s="46"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" ht="13.8">
       <c r="A13" s="39" t="s">
         <v>41</v>
       </c>
@@ -2453,7 +2459,7 @@
       </c>
       <c r="J13" s="46"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="13.8">
       <c r="A14" s="39" t="s">
         <v>44</v>
       </c>
@@ -2487,7 +2493,7 @@
       </c>
       <c r="J14" s="46"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" ht="13.8">
       <c r="A15" s="39" t="s">
         <v>44</v>
       </c>
@@ -2521,7 +2527,7 @@
       </c>
       <c r="J15" s="46"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" ht="13.8">
       <c r="A16" s="39" t="s">
         <v>44</v>
       </c>
@@ -2555,7 +2561,7 @@
       </c>
       <c r="J16" s="46"/>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" ht="13.8">
       <c r="A17" s="39" t="s">
         <v>44</v>
       </c>
@@ -2589,7 +2595,7 @@
       </c>
       <c r="J17" s="46"/>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" ht="13.8">
       <c r="A18" s="39" t="s">
         <v>48</v>
       </c>
@@ -2623,7 +2629,7 @@
       </c>
       <c r="J18" s="46"/>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" ht="13.8">
       <c r="A19" s="39" t="s">
         <v>48</v>
       </c>
@@ -2657,7 +2663,7 @@
       </c>
       <c r="J19" s="46"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" ht="13.8">
       <c r="A20" s="39" t="s">
         <v>48</v>
       </c>
@@ -2691,7 +2697,7 @@
       </c>
       <c r="J20" s="46"/>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" ht="13.8">
       <c r="A21" s="39" t="s">
         <v>48</v>
       </c>
@@ -2725,7 +2731,7 @@
       </c>
       <c r="J21" s="46"/>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" ht="13.8">
       <c r="A22" s="39" t="s">
         <v>53</v>
       </c>
@@ -2759,7 +2765,7 @@
       </c>
       <c r="J22" s="46"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" ht="13.8">
       <c r="A23" s="39" t="s">
         <v>53</v>
       </c>
@@ -2793,7 +2799,7 @@
       </c>
       <c r="J23" s="46"/>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" ht="13.8">
       <c r="A24" s="39" t="s">
         <v>53</v>
       </c>
@@ -2827,7 +2833,7 @@
       </c>
       <c r="J24" s="46"/>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" ht="13.8">
       <c r="A25" s="39" t="s">
         <v>56</v>
       </c>
@@ -2861,7 +2867,7 @@
       </c>
       <c r="J25" s="46"/>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" ht="13.8">
       <c r="A26" s="39" t="s">
         <v>56</v>
       </c>
@@ -2895,124 +2901,124 @@
       </c>
       <c r="J26" s="46"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" ht="13.2">
       <c r="B29" s="1"/>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" ht="13.2">
       <c r="A31" s="49"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" ht="13.2">
       <c r="B32" s="1"/>
       <c r="D32" s="1"/>
     </row>
-    <row r="33" spans="2:4">
+    <row r="33" spans="2:4" ht="13.2">
       <c r="B33" s="1"/>
       <c r="D33" s="1"/>
     </row>
-    <row r="34" spans="2:4">
+    <row r="34" spans="2:4" ht="13.8">
       <c r="B34" s="50"/>
       <c r="C34" s="50"/>
       <c r="D34" s="50"/>
     </row>
-    <row r="35" spans="2:4">
+    <row r="35" spans="2:4" ht="13.8">
       <c r="B35" s="47"/>
       <c r="C35" s="47"/>
       <c r="D35" s="47"/>
     </row>
-    <row r="36" spans="2:4">
+    <row r="36" spans="2:4" ht="13.8">
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="47"/>
     </row>
-    <row r="37" spans="2:4">
+    <row r="37" spans="2:4" ht="13.8">
       <c r="B37" s="47"/>
       <c r="C37" s="47"/>
       <c r="D37" s="47"/>
     </row>
-    <row r="38" spans="2:4">
+    <row r="38" spans="2:4" ht="13.8">
       <c r="B38" s="47"/>
       <c r="C38" s="47"/>
       <c r="D38" s="47"/>
     </row>
-    <row r="39" spans="2:4">
+    <row r="39" spans="2:4" ht="13.8">
       <c r="B39" s="47"/>
       <c r="C39" s="47"/>
       <c r="D39" s="47"/>
     </row>
-    <row r="40" spans="2:4">
+    <row r="40" spans="2:4" ht="13.8">
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="47"/>
     </row>
-    <row r="41" spans="2:4">
+    <row r="41" spans="2:4" ht="13.8">
       <c r="B41" s="47"/>
       <c r="C41" s="47"/>
       <c r="D41" s="47"/>
     </row>
-    <row r="42" spans="2:4">
+    <row r="42" spans="2:4" ht="13.8">
       <c r="B42" s="47"/>
       <c r="C42" s="47"/>
       <c r="D42" s="47"/>
     </row>
-    <row r="43" spans="2:4">
+    <row r="43" spans="2:4" ht="13.8">
       <c r="B43" s="47"/>
       <c r="C43" s="47"/>
       <c r="D43" s="47"/>
     </row>
-    <row r="44" spans="2:4">
+    <row r="44" spans="2:4" ht="13.8">
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="47"/>
     </row>
-    <row r="45" spans="2:4">
+    <row r="45" spans="2:4" ht="13.8">
       <c r="B45" s="47"/>
       <c r="C45" s="47"/>
       <c r="D45" s="47"/>
     </row>
-    <row r="46" spans="2:4">
+    <row r="46" spans="2:4" ht="13.8">
       <c r="B46" s="47"/>
       <c r="C46" s="47"/>
       <c r="D46" s="47"/>
     </row>
-    <row r="47" spans="2:4">
+    <row r="47" spans="2:4" ht="13.8">
       <c r="B47" s="47"/>
       <c r="C47" s="47"/>
       <c r="D47" s="47"/>
     </row>
-    <row r="48" spans="2:4">
+    <row r="48" spans="2:4" ht="13.8">
       <c r="B48" s="47"/>
       <c r="C48" s="47"/>
       <c r="D48" s="47"/>
     </row>
-    <row r="49" spans="2:4">
+    <row r="49" spans="2:4" ht="13.8">
       <c r="B49" s="47"/>
       <c r="C49" s="47"/>
       <c r="D49" s="47"/>
     </row>
-    <row r="50" spans="2:4">
+    <row r="50" spans="2:4" ht="13.8">
       <c r="B50" s="47"/>
       <c r="C50" s="47"/>
       <c r="D50" s="47"/>
     </row>
-    <row r="51" spans="2:4">
+    <row r="51" spans="2:4" ht="13.8">
       <c r="B51" s="47"/>
       <c r="C51" s="47"/>
       <c r="D51" s="47"/>
     </row>
-    <row r="52" spans="2:4">
+    <row r="52" spans="2:4" ht="13.8">
       <c r="B52" s="47"/>
       <c r="C52" s="47"/>
       <c r="D52" s="47"/>
     </row>
-    <row r="53" spans="2:4">
+    <row r="53" spans="2:4" ht="13.8">
       <c r="B53" s="47"/>
       <c r="C53" s="47"/>
       <c r="D53" s="47"/>
     </row>
-    <row r="54" spans="2:4">
+    <row r="54" spans="2:4" ht="13.8">
       <c r="B54" s="47"/>
       <c r="C54" s="47"/>
       <c r="D54" s="47"/>
@@ -3050,15 +3056,15 @@
   <dimension ref="B1:J22"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="2" max="2" width="29" style="73" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="75"/>
-    <col min="4" max="4" width="8.88671875" style="75" customWidth="1"/>
-    <col min="5" max="9" width="8.88671875" style="75"/>
-    <col min="10" max="10" width="10.77734375" style="71" customWidth="1"/>
+    <col min="2" max="2" width="29" style="64" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="66"/>
+    <col min="4" max="4" width="8.88671875" style="66" customWidth="1"/>
+    <col min="5" max="9" width="8.88671875" style="66"/>
+    <col min="10" max="10" width="10.77734375" style="63" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="64" t="s">
         <v>162</v>
       </c>
       <c r="C1" s="85" t="s">
@@ -3070,301 +3076,301 @@
       <c r="G1" s="85"/>
       <c r="H1" s="85"/>
       <c r="I1" s="85"/>
-      <c r="J1" s="67" t="s">
+      <c r="J1" s="59" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="2" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="76" t="s">
+      <c r="C2" s="67" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="68">
-        <v>14</v>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="60">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B3" s="72"/>
-      <c r="C3" s="78" t="s">
+      <c r="B3" s="84"/>
+      <c r="C3" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="69"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="61"/>
     </row>
     <row r="4" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B4" s="72"/>
-      <c r="C4" s="78" t="s">
+      <c r="B4" s="84"/>
+      <c r="C4" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="69"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="61"/>
     </row>
     <row r="5" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B5" s="72"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="84"/>
+      <c r="C5" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="D5" s="79"/>
-      <c r="E5" s="79"/>
-      <c r="F5" s="79"/>
-      <c r="G5" s="79"/>
-      <c r="H5" s="79"/>
-      <c r="I5" s="79"/>
-      <c r="J5" s="69"/>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="70"/>
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="61"/>
     </row>
     <row r="6" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B6" s="72"/>
-      <c r="C6" s="80" t="s">
+      <c r="B6" s="84"/>
+      <c r="C6" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="81"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="70"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="62"/>
     </row>
     <row r="7" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B7" s="72" t="s">
+      <c r="B7" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="82" t="s">
+      <c r="C7" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-      <c r="F7" s="79"/>
-      <c r="G7" s="79"/>
-      <c r="H7" s="79"/>
-      <c r="I7" s="79"/>
-      <c r="J7" s="68">
-        <v>7</v>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="70"/>
+      <c r="J7" s="60">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B8" s="72"/>
-      <c r="C8" s="82" t="s">
+      <c r="B8" s="84"/>
+      <c r="C8" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="79"/>
-      <c r="E8" s="79"/>
-      <c r="F8" s="79"/>
-      <c r="G8" s="79"/>
-      <c r="H8" s="79"/>
-      <c r="I8" s="79"/>
-      <c r="J8" s="70"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="70"/>
+      <c r="H8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="62"/>
     </row>
     <row r="9" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B9" s="72" t="s">
+      <c r="B9" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="83" t="s">
+      <c r="C9" s="74" t="s">
         <v>78</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="77"/>
-      <c r="F9" s="77"/>
-      <c r="G9" s="77"/>
-      <c r="H9" s="77"/>
-      <c r="I9" s="77"/>
-      <c r="J9" s="68">
-        <v>29</v>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
+      <c r="I9" s="68"/>
+      <c r="J9" s="60">
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B10" s="72"/>
-      <c r="C10" s="82" t="s">
+      <c r="B10" s="84"/>
+      <c r="C10" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="79"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="79"/>
-      <c r="I10" s="79"/>
-      <c r="J10" s="69"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="61"/>
     </row>
     <row r="11" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B11" s="72"/>
-      <c r="C11" s="82" t="s">
+      <c r="B11" s="84"/>
+      <c r="C11" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="79"/>
-      <c r="E11" s="79"/>
-      <c r="F11" s="79"/>
-      <c r="G11" s="79"/>
-      <c r="H11" s="79"/>
-      <c r="I11" s="79"/>
-      <c r="J11" s="69"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="70"/>
+      <c r="I11" s="70"/>
+      <c r="J11" s="61"/>
     </row>
     <row r="12" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B12" s="72"/>
-      <c r="C12" s="82" t="s">
+      <c r="B12" s="84"/>
+      <c r="C12" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="79"/>
-      <c r="E12" s="79"/>
-      <c r="F12" s="79"/>
-      <c r="G12" s="79"/>
-      <c r="H12" s="79"/>
-      <c r="I12" s="79"/>
-      <c r="J12" s="69"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="70"/>
+      <c r="H12" s="70"/>
+      <c r="I12" s="70"/>
+      <c r="J12" s="61"/>
     </row>
     <row r="13" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B13" s="72" t="s">
+      <c r="B13" s="84" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="83" t="s">
+      <c r="C13" s="74" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="77"/>
-      <c r="E13" s="77"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="77"/>
-      <c r="J13" s="68">
-        <v>7</v>
+      <c r="D13" s="68"/>
+      <c r="E13" s="68"/>
+      <c r="F13" s="68"/>
+      <c r="G13" s="68"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="68"/>
+      <c r="J13" s="60">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B14" s="72"/>
-      <c r="C14" s="82" t="s">
+      <c r="B14" s="84"/>
+      <c r="C14" s="73" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="79"/>
-      <c r="E14" s="79"/>
-      <c r="F14" s="79"/>
-      <c r="G14" s="79"/>
-      <c r="H14" s="79"/>
-      <c r="I14" s="79"/>
-      <c r="J14" s="69"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="70"/>
+      <c r="H14" s="70"/>
+      <c r="I14" s="70"/>
+      <c r="J14" s="61"/>
     </row>
     <row r="15" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B15" s="72"/>
-      <c r="C15" s="82" t="s">
+      <c r="B15" s="84"/>
+      <c r="C15" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="79"/>
-      <c r="E15" s="79"/>
-      <c r="F15" s="79"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="69"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="70"/>
+      <c r="G15" s="70"/>
+      <c r="H15" s="70"/>
+      <c r="I15" s="70"/>
+      <c r="J15" s="61"/>
     </row>
     <row r="16" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B16" s="72"/>
-      <c r="C16" s="82" t="s">
+      <c r="B16" s="84"/>
+      <c r="C16" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="79"/>
-      <c r="E16" s="79"/>
-      <c r="F16" s="79"/>
-      <c r="G16" s="79"/>
-      <c r="H16" s="79"/>
-      <c r="I16" s="79"/>
-      <c r="J16" s="69"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="70"/>
+      <c r="I16" s="70"/>
+      <c r="J16" s="61"/>
     </row>
     <row r="17" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B17" s="72" t="s">
+      <c r="B17" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="83" t="s">
+      <c r="C17" s="74" t="s">
         <v>86</v>
       </c>
-      <c r="D17" s="77"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="77"/>
-      <c r="J17" s="68">
-        <v>7</v>
+      <c r="D17" s="68"/>
+      <c r="E17" s="68"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="68"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="68"/>
+      <c r="J17" s="60">
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B18" s="72"/>
-      <c r="C18" s="82" t="s">
+      <c r="B18" s="84"/>
+      <c r="C18" s="73" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="79"/>
-      <c r="E18" s="79"/>
-      <c r="F18" s="79"/>
-      <c r="G18" s="79"/>
-      <c r="H18" s="79"/>
-      <c r="I18" s="79"/>
-      <c r="J18" s="69"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="70"/>
+      <c r="F18" s="70"/>
+      <c r="G18" s="70"/>
+      <c r="H18" s="70"/>
+      <c r="I18" s="70"/>
+      <c r="J18" s="61"/>
     </row>
     <row r="19" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B19" s="72"/>
-      <c r="C19" s="82" t="s">
+      <c r="B19" s="84"/>
+      <c r="C19" s="73" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
-      <c r="F19" s="79"/>
-      <c r="G19" s="79"/>
-      <c r="H19" s="79"/>
-      <c r="I19" s="79"/>
-      <c r="J19" s="69"/>
+      <c r="D19" s="70"/>
+      <c r="E19" s="70"/>
+      <c r="F19" s="70"/>
+      <c r="G19" s="70"/>
+      <c r="H19" s="70"/>
+      <c r="I19" s="70"/>
+      <c r="J19" s="61"/>
     </row>
     <row r="20" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B20" s="72" t="s">
+      <c r="B20" s="84" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="83" t="s">
+      <c r="C20" s="74" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="77"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="77"/>
-      <c r="G20" s="77"/>
-      <c r="H20" s="77"/>
-      <c r="I20" s="77"/>
-      <c r="J20" s="68">
-        <v>14</v>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="68"/>
+      <c r="J20" s="60">
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="16.8" customHeight="1">
-      <c r="B21" s="72"/>
-      <c r="C21" s="84" t="s">
+      <c r="B21" s="84"/>
+      <c r="C21" s="75" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="81"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="81"/>
-      <c r="G21" s="81"/>
-      <c r="H21" s="81"/>
-      <c r="I21" s="81"/>
-      <c r="J21" s="70"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="72"/>
+      <c r="F21" s="72"/>
+      <c r="G21" s="72"/>
+      <c r="H21" s="72"/>
+      <c r="I21" s="72"/>
+      <c r="J21" s="62"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="I22" s="75" t="s">
+      <c r="I22" s="66" t="s">
         <v>161</v>
       </c>
-      <c r="J22" s="74">
+      <c r="J22" s="65">
         <f>SUM(J2:J20)</f>
-        <v>78</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -3592,7 +3598,7 @@
     <col min="7" max="7" width="5.5546875" customWidth="1"/>
     <col min="8" max="9" width="17.5546875" customWidth="1"/>
     <col min="10" max="11" width="12.5546875" customWidth="1"/>
-    <col min="12" max="12" width="7.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>